<commit_message>
Actualizacao pagina de poupança
</commit_message>
<xml_diff>
--- a/Presencas_BPA.xlsx
+++ b/Presencas_BPA.xlsx
@@ -771,13 +771,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{231CD796-1286-4149-9814-B9BAAB97ABD8}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{AF7BA76C-0FDD-4220-918F-DD6FC409FB35}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{C3290A6A-414A-4B5C-99A0-4573CE488C6F}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3A20FF9D-0D47-40CA-8BCF-F9EE60D0F171}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5C1A7141-A43B-4492-BEC5-CBDE236BAAC6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{53AF1E20-F40E-4805-A2A9-F5BA51AF965A}"/>
 </file>
</xml_diff>